<commit_message>
Polish Supply & Absorption tab; begin-based UC rule; concession % rows
- Fix row heights (compact 14.4) on the Supply & Absorption tab.
- Remove the Cum. Unabsorbed row.
- Drive UNDER CONSTRUCTION vs PROPOSED by Construction Begin: ground broken
  (begin <= as-of) -> UC even if a source lags; future begin -> Proposed (still
  gets an estimated completion for the pipeline).
- Add subject Concession % row (historical from HelloData / CoStar) and relabel
  the forward concessions block as the editable % assumption.
- Sort each Competitive Analysis section chronologically (earliest first).
- Replace the inline reconciliation lines with a collapsed (grouped) detail
  section: rent source used per year (CoStar->HD) + UC-vs-CoStar reconciliation
  + partial-quarter note.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Canyon_Ridge__Supply_Chart.xlsx
+++ b/output/Canyon_Ridge__Supply_Chart.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0;;&quot;—&quot;"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,6 +91,11 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="FF000000"/>
       <sz val="8"/>
     </font>
@@ -251,9 +256,6 @@
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -270,9 +272,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -294,6 +293,9 @@
     <xf numFmtId="164" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -304,6 +306,7 @@
     <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -775,35 +778,39 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>The Mill at Loggers Creek</t>
+          <t>The Timbers at Harris Ranch</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>125</v>
+        <v>274</v>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Q2 2024</t>
+          <t>Q2 2023</t>
         </is>
       </c>
       <c r="F6" s="10" t="n">
-        <v>0.92</v>
+        <v>0.967153</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>2104</v>
+        <v>2196</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Baron Properties</t>
+          <t>Highland Canyon Partners</t>
         </is>
       </c>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
-        </is>
-      </c>
-      <c r="K6" s="8" t="n"/>
+          <t>Garden</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Year built: 2023/2024; Occ: CoStar 97% vs RealPage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="7" t="n">
@@ -851,39 +858,35 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>The Timbers at Harris Ranch</t>
+          <t>The Mill at Loggers Creek</t>
         </is>
       </c>
       <c r="D8" s="9" t="n">
-        <v>274</v>
+        <v>125</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Q2 2023</t>
+          <t>Q2 2024</t>
         </is>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0.967153</v>
+        <v>0.92</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>2196</v>
+        <v>2104</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Highland Canyon Partners</t>
+          <t>Baron Properties</t>
         </is>
       </c>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>Garden</t>
-        </is>
-      </c>
-      <c r="K8" s="8" t="inlineStr">
-        <is>
-          <t>Year built: 2023/2024; Occ: CoStar 97% vs RealPage 100%</t>
-        </is>
-      </c>
+          <t>Mid-Rise</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="12" t="n"/>
@@ -899,15 +902,15 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>Vista Point</t>
+          <t>Harris Ranch East</t>
         </is>
       </c>
       <c r="D11" s="16" t="n">
-        <v>893</v>
+        <v>59</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Q2 2028</t>
+          <t>Q4 2026</t>
         </is>
       </c>
       <c r="F11" s="17" t="n"/>
@@ -924,7 +927,7 @@
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Single Family</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
@@ -939,15 +942,15 @@
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>3300 South Vista Avenue</t>
+          <t>Station Village</t>
         </is>
       </c>
       <c r="D12" s="16" t="n">
-        <v>180</v>
+        <v>84</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Q1 2028</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="F12" s="17" t="n"/>
@@ -958,13 +961,13 @@
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Privately Owned</t>
         </is>
       </c>
       <c r="I12" s="14" t="n"/>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K12" s="15" t="inlineStr">
@@ -979,15 +982,15 @@
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>Seasons on the Bench</t>
+          <t>1519 South Londoner Avenue</t>
         </is>
       </c>
       <c r="D13" s="16" t="n">
-        <v>358</v>
+        <v>189</v>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Q4 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="F13" s="17" t="n"/>
@@ -1019,15 +1022,15 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>1519 South Londoner Avenue</t>
+          <t>Seasons on the Bench</t>
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>189</v>
+        <v>358</v>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Q3 2027</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="F14" s="17" t="n"/>
@@ -1059,15 +1062,15 @@
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Station Village</t>
+          <t>3300 South Vista Avenue</t>
         </is>
       </c>
       <c r="D15" s="16" t="n">
-        <v>84</v>
+        <v>180</v>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q1 2028</t>
         </is>
       </c>
       <c r="F15" s="17" t="n"/>
@@ -1078,13 +1081,13 @@
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>Privately Owned</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I15" s="14" t="n"/>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K15" s="15" t="inlineStr">
@@ -1099,15 +1102,15 @@
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Harris Ranch East</t>
+          <t>Vista Point</t>
         </is>
       </c>
       <c r="D16" s="16" t="n">
-        <v>59</v>
+        <v>893</v>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Q4 2026</t>
+          <t>Q2 2028</t>
         </is>
       </c>
       <c r="F16" s="17" t="n"/>
@@ -1124,7 +1127,7 @@
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>Single Family</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K16" s="15" t="inlineStr">
@@ -1155,10 +1158,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Z52"/>
+  <dimension ref="B1:Z60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1179,19 +1182,19 @@
     <col width="28" customWidth="1" min="18" max="18"/>
     <col width="7" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="9" customWidth="1" min="21" max="21"/>
     <col hidden="1" width="8" customWidth="1" min="22" max="22"/>
     <col hidden="1" width="7" customWidth="1" min="23" max="23"/>
     <col hidden="1" width="6" customWidth="1" min="24" max="24"/>
     <col hidden="1" width="13" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="14.4" customHeight="1">
       <c r="Z1" t="n">
         <v>8105</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
+    <row r="2" ht="20" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
           <t>SUPPLY &amp; ABSORPTION  —  5-MILE MARKET (relative-year / TTM)</t>
@@ -1202,7 +1205,7 @@
         <v/>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="14.4" customHeight="1">
       <c r="R3" s="20" t="inlineStr">
         <is>
           <t>UNDER CONSTRUCTION (linked from Competitive Analysis)</t>
@@ -1213,7 +1216,7 @@
         <v/>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="14.4" customHeight="1">
       <c r="B4" s="21" t="inlineStr">
         <is>
           <t>As-of Quarter</t>
@@ -1240,7 +1243,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="14.4" customHeight="1">
       <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Close Quarter (Y1 start)</t>
@@ -1252,7 +1255,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="14.4" customHeight="1">
       <c r="B6" s="21" t="inlineStr">
         <is>
           <t>Stabilization Target</t>
@@ -1262,7 +1265,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="14.4" customHeight="1">
       <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Demand Scenario</t>
@@ -1279,7 +1282,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="14.4" customHeight="1">
       <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Bear Annual Absorption</t>
@@ -1309,7 +1312,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="14.4" customHeight="1">
       <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Base Annual Absorption</t>
@@ -1349,7 +1352,7 @@
         <v/>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="14.4" customHeight="1">
       <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Bull Annual Absorption</t>
@@ -1389,7 +1392,7 @@
         <v/>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="14.4" customHeight="1">
       <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Selected Annual Demand</t>
@@ -1430,17 +1433,7 @@
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="21" t="inlineStr">
-        <is>
-          <t>UC scheduled vs CoStar UC</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>0 / 27</t>
-        </is>
-      </c>
+    <row r="12" ht="14.4" customHeight="1">
       <c r="R12" s="27" t="inlineStr">
         <is>
           <t>3300 South Vista Avenue</t>
@@ -1472,17 +1465,7 @@
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="21" t="inlineStr">
-        <is>
-          <t>Subject rent source</t>
-        </is>
-      </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+    <row r="13" ht="14.4" customHeight="1">
       <c r="R13" s="27" t="inlineStr">
         <is>
           <t>Station Village</t>
@@ -1514,7 +1497,7 @@
         <v/>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="14.4" customHeight="1">
       <c r="R14" s="27" t="inlineStr">
         <is>
           <t>Harris Ranch East</t>
@@ -1546,7 +1529,9 @@
         <v/>
       </c>
     </row>
-    <row r="17">
+    <row r="15" ht="14.4" customHeight="1"/>
+    <row r="16" ht="14.4" customHeight="1"/>
+    <row r="17" ht="14.4" customHeight="1">
       <c r="B17" s="21" t="inlineStr">
         <is>
           <t>5-MILE MARKET</t>
@@ -1587,426 +1572,396 @@
           <t>Y0</t>
         </is>
       </c>
-      <c r="J17" s="32" t="inlineStr">
+      <c r="J17" s="31" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="K17" s="32" t="inlineStr">
+      <c r="K17" s="31" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="L17" s="32" t="inlineStr">
+      <c r="L17" s="31" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="M17" s="32" t="inlineStr">
+      <c r="M17" s="31" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="N17" s="32" t="inlineStr">
+      <c r="N17" s="31" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="O17" s="32" t="inlineStr">
+      <c r="O17" s="31" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="C18" s="33" t="inlineStr">
-        <is>
-          <t>Q3 2019–Q2 2020</t>
-        </is>
-      </c>
-      <c r="D18" s="33" t="inlineStr">
-        <is>
-          <t>Q3 2020–Q2 2021</t>
-        </is>
-      </c>
-      <c r="E18" s="33" t="inlineStr">
-        <is>
-          <t>Q3 2021–Q2 2022</t>
-        </is>
-      </c>
-      <c r="F18" s="33" t="inlineStr">
-        <is>
-          <t>Q3 2022–Q2 2023</t>
-        </is>
-      </c>
-      <c r="G18" s="33" t="inlineStr">
-        <is>
-          <t>Q3 2023–Q2 2024</t>
-        </is>
-      </c>
-      <c r="H18" s="33" t="inlineStr">
-        <is>
-          <t>Q3 2024–Q2 2025</t>
-        </is>
-      </c>
-      <c r="I18" s="33" t="inlineStr">
-        <is>
-          <t>Q3 2025–Q2 2026</t>
-        </is>
-      </c>
-      <c r="J18" s="33" t="inlineStr">
+    <row r="18" ht="14.4" customHeight="1">
+      <c r="C18" s="32" t="inlineStr">
+        <is>
+          <t>Q3'19-Q2'20</t>
+        </is>
+      </c>
+      <c r="D18" s="32" t="inlineStr">
+        <is>
+          <t>Q3'20-Q2'21</t>
+        </is>
+      </c>
+      <c r="E18" s="32" t="inlineStr">
+        <is>
+          <t>Q3'21-Q2'22</t>
+        </is>
+      </c>
+      <c r="F18" s="32" t="inlineStr">
+        <is>
+          <t>Q3'22-Q2'23</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="inlineStr">
+        <is>
+          <t>Q3'23-Q2'24</t>
+        </is>
+      </c>
+      <c r="H18" s="32" t="inlineStr">
+        <is>
+          <t>Q3'24-Q2'25</t>
+        </is>
+      </c>
+      <c r="I18" s="32" t="inlineStr">
+        <is>
+          <t>Q3'25-Q2'26</t>
+        </is>
+      </c>
+      <c r="J18" s="32" t="inlineStr">
         <is>
           <t>Hold Yr 1</t>
         </is>
       </c>
-      <c r="K18" s="33" t="inlineStr">
+      <c r="K18" s="32" t="inlineStr">
         <is>
           <t>Hold Yr 2</t>
         </is>
       </c>
-      <c r="L18" s="33" t="inlineStr">
+      <c r="L18" s="32" t="inlineStr">
         <is>
           <t>Hold Yr 3</t>
         </is>
       </c>
-      <c r="M18" s="33" t="inlineStr">
+      <c r="M18" s="32" t="inlineStr">
         <is>
           <t>Hold Yr 4</t>
         </is>
       </c>
-      <c r="N18" s="33" t="inlineStr">
+      <c r="N18" s="32" t="inlineStr">
         <is>
           <t>Hold Yr 5</t>
         </is>
       </c>
-      <c r="O18" s="33" t="inlineStr">
+      <c r="O18" s="32" t="inlineStr">
         <is>
           <t>Hold Yr 6</t>
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="14.4" customHeight="1">
       <c r="B19" s="21" t="inlineStr">
         <is>
           <t>NEW SUPPLY (5-mi)</t>
         </is>
       </c>
-      <c r="C19" s="34" t="n">
+      <c r="C19" s="33" t="n">
         <v>213</v>
       </c>
-      <c r="D19" s="34" t="n">
+      <c r="D19" s="33" t="n">
         <v>237</v>
       </c>
-      <c r="E19" s="34" t="n">
+      <c r="E19" s="33" t="n">
         <v>33</v>
       </c>
-      <c r="F19" s="34" t="n">
+      <c r="F19" s="33" t="n">
         <v>289</v>
       </c>
-      <c r="G19" s="34" t="n">
+      <c r="G19" s="33" t="n">
         <v>178</v>
       </c>
-      <c r="H19" s="34" t="n">
+      <c r="H19" s="33" t="n">
         <v>334</v>
       </c>
-      <c r="I19" s="34" t="n">
+      <c r="I19" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="J19" s="35">
+      <c r="J19" s="34">
         <f>SUMIFS($S$5:$S$5,$W$5:$W$5,1)+SUMIFS($S$9:$S$14,$W$9:$W$14,1,$X$9:$X$14,1)</f>
         <v/>
       </c>
-      <c r="K19" s="35">
+      <c r="K19" s="34">
         <f>SUMIFS($S$5:$S$5,$W$5:$W$5,2)+SUMIFS($S$9:$S$14,$W$9:$W$14,2,$X$9:$X$14,1)</f>
         <v/>
       </c>
-      <c r="L19" s="35">
+      <c r="L19" s="34">
         <f>SUMIFS($S$5:$S$5,$W$5:$W$5,3)+SUMIFS($S$9:$S$14,$W$9:$W$14,3,$X$9:$X$14,1)</f>
         <v/>
       </c>
-      <c r="M19" s="35">
+      <c r="M19" s="34">
         <f>SUMIFS($S$5:$S$5,$W$5:$W$5,4)+SUMIFS($S$9:$S$14,$W$9:$W$14,4,$X$9:$X$14,1)</f>
         <v/>
       </c>
-      <c r="N19" s="35">
+      <c r="N19" s="34">
         <f>SUMIFS($S$5:$S$5,$W$5:$W$5,5)+SUMIFS($S$9:$S$14,$W$9:$W$14,5,$X$9:$X$14,1)</f>
         <v/>
       </c>
-      <c r="O19" s="35">
+      <c r="O19" s="34">
         <f>SUMIFS($S$5:$S$5,$W$5:$W$5,6)+SUMIFS($S$9:$S$14,$W$9:$W$14,6,$X$9:$X$14,1)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="14.4" customHeight="1">
       <c r="B20" s="21" t="inlineStr">
         <is>
           <t>ABSORPTION (5-mi)</t>
         </is>
       </c>
-      <c r="C20" s="34" t="n">
+      <c r="C20" s="33" t="n">
         <v>213</v>
       </c>
-      <c r="D20" s="34" t="n">
+      <c r="D20" s="33" t="n">
         <v>150</v>
       </c>
-      <c r="E20" s="34" t="n">
+      <c r="E20" s="33" t="n">
         <v>86</v>
       </c>
-      <c r="F20" s="34" t="n">
+      <c r="F20" s="33" t="n">
         <v>-91</v>
       </c>
-      <c r="G20" s="34" t="n">
+      <c r="G20" s="33" t="n">
         <v>277</v>
       </c>
-      <c r="H20" s="34" t="n">
+      <c r="H20" s="33" t="n">
         <v>399</v>
       </c>
-      <c r="I20" s="34" t="n">
+      <c r="I20" s="33" t="n">
         <v>216</v>
       </c>
-      <c r="J20" s="35">
+      <c r="J20" s="34">
         <f>J31-I31</f>
         <v/>
       </c>
-      <c r="K20" s="35">
+      <c r="K20" s="34">
         <f>K31-J31</f>
         <v/>
       </c>
-      <c r="L20" s="35">
+      <c r="L20" s="34">
         <f>L31-K31</f>
         <v/>
       </c>
-      <c r="M20" s="35">
+      <c r="M20" s="34">
         <f>M31-L31</f>
         <v/>
       </c>
-      <c r="N20" s="35">
+      <c r="N20" s="34">
         <f>N31-M31</f>
         <v/>
       </c>
-      <c r="O20" s="35">
+      <c r="O20" s="34">
         <f>O31-N31</f>
         <v/>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="14.4" customHeight="1">
       <c r="B21" s="21" t="inlineStr">
         <is>
           <t>OCCUPANCY (5-mi)</t>
         </is>
       </c>
-      <c r="C21" s="36" t="n">
+      <c r="C21" s="35" t="n">
         <v>0.968</v>
       </c>
-      <c r="D21" s="36" t="n">
+      <c r="D21" s="35" t="n">
         <v>0.953</v>
       </c>
-      <c r="E21" s="36" t="n">
+      <c r="E21" s="35" t="n">
         <v>0.963</v>
       </c>
-      <c r="F21" s="36" t="n">
+      <c r="F21" s="35" t="n">
         <v>0.895</v>
       </c>
-      <c r="G21" s="36" t="n">
+      <c r="G21" s="35" t="n">
         <v>0.916</v>
       </c>
-      <c r="H21" s="36" t="n">
+      <c r="H21" s="35" t="n">
         <v>0.9320000000000001</v>
       </c>
-      <c r="I21" s="36" t="n">
+      <c r="I21" s="35" t="n">
         <v>0.967</v>
       </c>
-      <c r="J21" s="37">
+      <c r="J21" s="36">
         <f>IFERROR(J31/J30,0)</f>
         <v/>
       </c>
-      <c r="K21" s="37">
+      <c r="K21" s="36">
         <f>IFERROR(K31/K30,0)</f>
         <v/>
       </c>
-      <c r="L21" s="37">
+      <c r="L21" s="36">
         <f>IFERROR(L31/L30,0)</f>
         <v/>
       </c>
-      <c r="M21" s="37">
+      <c r="M21" s="36">
         <f>IFERROR(M31/M30,0)</f>
         <v/>
       </c>
-      <c r="N21" s="37">
+      <c r="N21" s="36">
         <f>IFERROR(N31/N30,0)</f>
         <v/>
       </c>
-      <c r="O21" s="37">
+      <c r="O21" s="36">
         <f>IFERROR(O31/O30,0)</f>
         <v/>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="14.4" customHeight="1">
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>CUM. UNABSORBED (since -Y3)</t>
-        </is>
-      </c>
-      <c r="C22" s="38" t="n"/>
-      <c r="D22" s="38" t="n"/>
-      <c r="E22" s="38" t="n"/>
-      <c r="F22" s="38">
-        <f>F19-F20</f>
-        <v/>
-      </c>
-      <c r="G22" s="38">
-        <f>F22+G19-G20</f>
-        <v/>
-      </c>
-      <c r="H22" s="38">
-        <f>G22+H19-H20</f>
-        <v/>
-      </c>
-      <c r="I22" s="38">
-        <f>H22+I19-I20</f>
-        <v/>
-      </c>
-      <c r="J22" s="38">
-        <f>I22+J19-J20</f>
-        <v/>
-      </c>
-      <c r="K22" s="38">
-        <f>J22+K19-K20</f>
-        <v/>
-      </c>
-      <c r="L22" s="38">
-        <f>K22+L19-L20</f>
-        <v/>
-      </c>
-      <c r="M22" s="38">
-        <f>L22+M19-M20</f>
-        <v/>
-      </c>
-      <c r="N22" s="38">
-        <f>M22+N19-N20</f>
-        <v/>
-      </c>
-      <c r="O22" s="38">
-        <f>N22+O19-O20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
+          <t>SUBJECT (Canyon Ridge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="14.4" customHeight="1">
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>SUBJECT (Canyon Ridge)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="21" t="inlineStr">
-        <is>
           <t xml:space="preserve">  Market Rent  (CoStar→HD)</t>
         </is>
       </c>
-      <c r="C24" s="39" t="n"/>
-      <c r="D24" s="39" t="n"/>
-      <c r="E24" s="39" t="n"/>
-      <c r="F24" s="39" t="n"/>
-      <c r="G24" s="39" t="n"/>
-      <c r="H24" s="39" t="n"/>
-      <c r="I24" s="39" t="n"/>
-      <c r="J24" s="40" t="n"/>
-      <c r="K24" s="40" t="n"/>
-      <c r="L24" s="40" t="n"/>
-      <c r="M24" s="40" t="n"/>
-      <c r="N24" s="40" t="n"/>
-      <c r="O24" s="40" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="41" t="inlineStr">
+      <c r="C23" s="37" t="n"/>
+      <c r="D23" s="37" t="n"/>
+      <c r="E23" s="37" t="n"/>
+      <c r="F23" s="37" t="n"/>
+      <c r="G23" s="37" t="n"/>
+      <c r="H23" s="37" t="n"/>
+      <c r="I23" s="37" t="n"/>
+      <c r="J23" s="38" t="n"/>
+      <c r="K23" s="38" t="n"/>
+      <c r="L23" s="38" t="n"/>
+      <c r="M23" s="38" t="n"/>
+      <c r="N23" s="38" t="n"/>
+      <c r="O23" s="38" t="n"/>
+    </row>
+    <row r="24" ht="14.4" customHeight="1">
+      <c r="B24" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">    Market Rent YoY %</t>
         </is>
       </c>
-      <c r="C25" s="42" t="n"/>
-      <c r="D25" s="42">
-        <f>IFERROR(D24/C24-1,"")</f>
-        <v/>
-      </c>
-      <c r="E25" s="42">
-        <f>IFERROR(E24/D24-1,"")</f>
-        <v/>
-      </c>
-      <c r="F25" s="42">
-        <f>IFERROR(F24/E24-1,"")</f>
-        <v/>
-      </c>
-      <c r="G25" s="42">
-        <f>IFERROR(G24/F24-1,"")</f>
-        <v/>
-      </c>
-      <c r="H25" s="42">
-        <f>IFERROR(H24/G24-1,"")</f>
-        <v/>
-      </c>
-      <c r="I25" s="42">
-        <f>IFERROR(I24/H24-1,"")</f>
-        <v/>
-      </c>
-      <c r="J25" s="43" t="n"/>
-      <c r="K25" s="43" t="n"/>
-      <c r="L25" s="43" t="n"/>
-      <c r="M25" s="43" t="n"/>
-      <c r="N25" s="43" t="n"/>
-      <c r="O25" s="43" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="21" t="inlineStr">
+      <c r="C24" s="40" t="n"/>
+      <c r="D24" s="40">
+        <f>IFERROR(D23/C23-1,"")</f>
+        <v/>
+      </c>
+      <c r="E24" s="40">
+        <f>IFERROR(E23/D23-1,"")</f>
+        <v/>
+      </c>
+      <c r="F24" s="40">
+        <f>IFERROR(F23/E23-1,"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="40">
+        <f>IFERROR(G23/F23-1,"")</f>
+        <v/>
+      </c>
+      <c r="H24" s="40">
+        <f>IFERROR(H23/G23-1,"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="40">
+        <f>IFERROR(I23/H23-1,"")</f>
+        <v/>
+      </c>
+      <c r="J24" s="41" t="n"/>
+      <c r="K24" s="41" t="n"/>
+      <c r="L24" s="41" t="n"/>
+      <c r="M24" s="41" t="n"/>
+      <c r="N24" s="41" t="n"/>
+      <c r="O24" s="41" t="n"/>
+    </row>
+    <row r="25" ht="14.4" customHeight="1">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  Effective Rent</t>
         </is>
       </c>
-      <c r="C26" s="39" t="n"/>
-      <c r="D26" s="39" t="n"/>
-      <c r="E26" s="39" t="n"/>
-      <c r="F26" s="39" t="n"/>
-      <c r="G26" s="39" t="n"/>
-      <c r="H26" s="39" t="n"/>
-      <c r="I26" s="39" t="n"/>
-      <c r="J26" s="40" t="n"/>
-      <c r="K26" s="40" t="n"/>
-      <c r="L26" s="40" t="n"/>
-      <c r="M26" s="40" t="n"/>
-      <c r="N26" s="40" t="n"/>
-      <c r="O26" s="40" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="41" t="inlineStr">
+      <c r="C25" s="37" t="n"/>
+      <c r="D25" s="37" t="n"/>
+      <c r="E25" s="37" t="n"/>
+      <c r="F25" s="37" t="n"/>
+      <c r="G25" s="37" t="n"/>
+      <c r="H25" s="37" t="n"/>
+      <c r="I25" s="37" t="n"/>
+      <c r="J25" s="38" t="n"/>
+      <c r="K25" s="38" t="n"/>
+      <c r="L25" s="38" t="n"/>
+      <c r="M25" s="38" t="n"/>
+      <c r="N25" s="38" t="n"/>
+      <c r="O25" s="38" t="n"/>
+    </row>
+    <row r="26" ht="14.4" customHeight="1">
+      <c r="B26" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">    Effective Rent YoY %</t>
         </is>
       </c>
+      <c r="C26" s="40" t="n"/>
+      <c r="D26" s="40">
+        <f>IFERROR(D25/C25-1,"")</f>
+        <v/>
+      </c>
+      <c r="E26" s="40">
+        <f>IFERROR(E25/D25-1,"")</f>
+        <v/>
+      </c>
+      <c r="F26" s="40">
+        <f>IFERROR(F25/E25-1,"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="40">
+        <f>IFERROR(G25/F25-1,"")</f>
+        <v/>
+      </c>
+      <c r="H26" s="40">
+        <f>IFERROR(H25/G25-1,"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="40">
+        <f>IFERROR(I25/H25-1,"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="41" t="n"/>
+      <c r="K26" s="41" t="n"/>
+      <c r="L26" s="41" t="n"/>
+      <c r="M26" s="41" t="n"/>
+      <c r="N26" s="41" t="n"/>
+      <c r="O26" s="41" t="n"/>
+    </row>
+    <row r="27" ht="14.4" customHeight="1">
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Occupancy (financials / CoStar)</t>
+        </is>
+      </c>
       <c r="C27" s="42" t="n"/>
-      <c r="D27" s="42">
-        <f>IFERROR(D26/C26-1,"")</f>
-        <v/>
-      </c>
-      <c r="E27" s="42">
-        <f>IFERROR(E26/D26-1,"")</f>
-        <v/>
-      </c>
-      <c r="F27" s="42">
-        <f>IFERROR(F26/E26-1,"")</f>
-        <v/>
-      </c>
-      <c r="G27" s="42">
-        <f>IFERROR(G26/F26-1,"")</f>
-        <v/>
-      </c>
-      <c r="H27" s="42">
-        <f>IFERROR(H26/G26-1,"")</f>
-        <v/>
-      </c>
-      <c r="I27" s="42">
-        <f>IFERROR(I26/H26-1,"")</f>
-        <v/>
-      </c>
+      <c r="D27" s="42" t="n"/>
+      <c r="E27" s="42" t="n"/>
+      <c r="F27" s="42" t="n"/>
+      <c r="G27" s="42" t="n"/>
+      <c r="H27" s="42" t="n"/>
+      <c r="I27" s="42" t="n"/>
       <c r="J27" s="43" t="n"/>
       <c r="K27" s="43" t="n"/>
       <c r="L27" s="43" t="n"/>
@@ -2014,575 +1969,670 @@
       <c r="N27" s="43" t="n"/>
       <c r="O27" s="43" t="n"/>
     </row>
-    <row r="28">
+    <row r="28" ht="14.4" customHeight="1">
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Occupancy (financials / CoStar)</t>
-        </is>
-      </c>
-      <c r="C28" s="44" t="n"/>
-      <c r="D28" s="44" t="n"/>
-      <c r="E28" s="44" t="n"/>
-      <c r="F28" s="44" t="n"/>
-      <c r="G28" s="44" t="n"/>
-      <c r="H28" s="44" t="n"/>
-      <c r="I28" s="44" t="n"/>
-      <c r="J28" s="45" t="n"/>
-      <c r="K28" s="45" t="n"/>
-      <c r="L28" s="45" t="n"/>
-      <c r="M28" s="45" t="n"/>
-      <c r="N28" s="45" t="n"/>
-      <c r="O28" s="45" t="n"/>
-    </row>
-    <row r="30" hidden="1">
+          <t xml:space="preserve">  Concession %</t>
+        </is>
+      </c>
+      <c r="C28" s="42" t="n"/>
+      <c r="D28" s="42" t="n"/>
+      <c r="E28" s="42" t="n"/>
+      <c r="F28" s="42" t="n"/>
+      <c r="G28" s="42" t="n"/>
+      <c r="H28" s="42" t="n"/>
+      <c r="I28" s="42" t="n"/>
+      <c r="J28" s="43" t="n"/>
+      <c r="K28" s="43" t="n"/>
+      <c r="L28" s="43" t="n"/>
+      <c r="M28" s="43" t="n"/>
+      <c r="N28" s="43" t="n"/>
+      <c r="O28" s="43" t="n"/>
+    </row>
+    <row r="29" ht="14.4" customHeight="1"/>
+    <row r="30" hidden="1" ht="14.4" customHeight="1">
       <c r="B30" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  inventory</t>
         </is>
       </c>
-      <c r="C30" s="38" t="n">
+      <c r="C30" s="44" t="n">
         <v>4845</v>
       </c>
-      <c r="D30" s="38" t="n">
+      <c r="D30" s="44" t="n">
         <v>5082</v>
       </c>
-      <c r="E30" s="38" t="n">
+      <c r="E30" s="44" t="n">
         <v>5115</v>
       </c>
-      <c r="F30" s="38" t="n">
+      <c r="F30" s="44" t="n">
         <v>5404</v>
       </c>
-      <c r="G30" s="38" t="n">
+      <c r="G30" s="44" t="n">
         <v>5582</v>
       </c>
-      <c r="H30" s="38" t="n">
+      <c r="H30" s="44" t="n">
         <v>5916</v>
       </c>
-      <c r="I30" s="38" t="n">
+      <c r="I30" s="44" t="n">
         <v>5925</v>
       </c>
-      <c r="J30" s="38">
+      <c r="J30" s="44">
         <f>I30+J19</f>
         <v/>
       </c>
-      <c r="K30" s="38">
+      <c r="K30" s="44">
         <f>J30+K19</f>
         <v/>
       </c>
-      <c r="L30" s="38">
+      <c r="L30" s="44">
         <f>K30+L19</f>
         <v/>
       </c>
-      <c r="M30" s="38">
+      <c r="M30" s="44">
         <f>L30+M19</f>
         <v/>
       </c>
-      <c r="N30" s="38">
+      <c r="N30" s="44">
         <f>M30+N19</f>
         <v/>
       </c>
-      <c r="O30" s="38">
+      <c r="O30" s="44">
         <f>N30+O19</f>
         <v/>
       </c>
     </row>
-    <row r="31" hidden="1">
+    <row r="31" hidden="1" ht="14.4" customHeight="1">
       <c r="B31" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  occupied</t>
         </is>
       </c>
-      <c r="C31" s="38" t="n">
+      <c r="C31" s="44" t="n">
         <v>4691</v>
       </c>
-      <c r="D31" s="38" t="n">
+      <c r="D31" s="44" t="n">
         <v>4841</v>
       </c>
-      <c r="E31" s="38" t="n">
+      <c r="E31" s="44" t="n">
         <v>4927</v>
       </c>
-      <c r="F31" s="38" t="n">
+      <c r="F31" s="44" t="n">
         <v>4836</v>
       </c>
-      <c r="G31" s="38" t="n">
+      <c r="G31" s="44" t="n">
         <v>5113</v>
       </c>
-      <c r="H31" s="38" t="n">
+      <c r="H31" s="44" t="n">
         <v>5512</v>
       </c>
-      <c r="I31" s="38" t="n">
+      <c r="I31" s="44" t="n">
         <v>5727</v>
       </c>
-      <c r="J31" s="38">
+      <c r="J31" s="44">
         <f>MIN($C$6*J30,I31+$C$11)</f>
         <v/>
       </c>
-      <c r="K31" s="38">
+      <c r="K31" s="44">
         <f>MIN($C$6*K30,J31+$C$11)</f>
         <v/>
       </c>
-      <c r="L31" s="38">
+      <c r="L31" s="44">
         <f>MIN($C$6*L30,K31+$C$11)</f>
         <v/>
       </c>
-      <c r="M31" s="38">
+      <c r="M31" s="44">
         <f>MIN($C$6*M30,L31+$C$11)</f>
         <v/>
       </c>
-      <c r="N31" s="38">
+      <c r="N31" s="44">
         <f>MIN($C$6*N30,M31+$C$11)</f>
         <v/>
       </c>
-      <c r="O31" s="38">
+      <c r="O31" s="44">
         <f>MIN($C$6*O30,N31+$C$11)</f>
         <v/>
       </c>
     </row>
-    <row r="33">
+    <row r="32" ht="14.4" customHeight="1"/>
+    <row r="33" ht="14.4" customHeight="1">
       <c r="B33" s="21" t="inlineStr">
         <is>
           <t>IMPLIED 5-MI OCCUPANCY BY DEMAND SCENARIO</t>
         </is>
       </c>
-      <c r="J33" s="46" t="inlineStr">
+      <c r="J33" s="45" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="K33" s="46" t="inlineStr">
+      <c r="K33" s="45" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="L33" s="46" t="inlineStr">
+      <c r="L33" s="45" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="M33" s="46" t="inlineStr">
+      <c r="M33" s="45" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="N33" s="46" t="inlineStr">
+      <c r="N33" s="45" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="O33" s="46" t="inlineStr">
+      <c r="O33" s="45" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="14.4" customHeight="1">
       <c r="B34" s="21" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J34" s="47">
+      <c r="J34" s="46">
         <f>MIN($C$6,($I$31+$C$8*1)/J30)</f>
         <v/>
       </c>
-      <c r="K34" s="47">
+      <c r="K34" s="46">
         <f>MIN($C$6,($I$31+$C$8*2)/K30)</f>
         <v/>
       </c>
-      <c r="L34" s="47">
+      <c r="L34" s="46">
         <f>MIN($C$6,($I$31+$C$8*3)/L30)</f>
         <v/>
       </c>
-      <c r="M34" s="47">
+      <c r="M34" s="46">
         <f>MIN($C$6,($I$31+$C$8*4)/M30)</f>
         <v/>
       </c>
-      <c r="N34" s="47">
+      <c r="N34" s="46">
         <f>MIN($C$6,($I$31+$C$8*5)/N30)</f>
         <v/>
       </c>
-      <c r="O34" s="47">
+      <c r="O34" s="46">
         <f>MIN($C$6,($I$31+$C$8*6)/O30)</f>
         <v/>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="14.4" customHeight="1">
       <c r="B35" s="21" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J35" s="47">
+      <c r="J35" s="46">
         <f>MIN($C$6,($I$31+$C$9*1)/J30)</f>
         <v/>
       </c>
-      <c r="K35" s="47">
+      <c r="K35" s="46">
         <f>MIN($C$6,($I$31+$C$9*2)/K30)</f>
         <v/>
       </c>
-      <c r="L35" s="47">
+      <c r="L35" s="46">
         <f>MIN($C$6,($I$31+$C$9*3)/L30)</f>
         <v/>
       </c>
-      <c r="M35" s="47">
+      <c r="M35" s="46">
         <f>MIN($C$6,($I$31+$C$9*4)/M30)</f>
         <v/>
       </c>
-      <c r="N35" s="47">
+      <c r="N35" s="46">
         <f>MIN($C$6,($I$31+$C$9*5)/N30)</f>
         <v/>
       </c>
-      <c r="O35" s="47">
+      <c r="O35" s="46">
         <f>MIN($C$6,($I$31+$C$9*6)/O30)</f>
         <v/>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="14.4" customHeight="1">
       <c r="B36" s="21" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J36" s="47">
+      <c r="J36" s="46">
         <f>MIN($C$6,($I$31+$C$10*1)/J30)</f>
         <v/>
       </c>
-      <c r="K36" s="47">
+      <c r="K36" s="46">
         <f>MIN($C$6,($I$31+$C$10*2)/K30)</f>
         <v/>
       </c>
-      <c r="L36" s="47">
+      <c r="L36" s="46">
         <f>MIN($C$6,($I$31+$C$10*3)/L30)</f>
         <v/>
       </c>
-      <c r="M36" s="47">
+      <c r="M36" s="46">
         <f>MIN($C$6,($I$31+$C$10*4)/M30)</f>
         <v/>
       </c>
-      <c r="N36" s="47">
+      <c r="N36" s="46">
         <f>MIN($C$6,($I$31+$C$10*5)/N30)</f>
         <v/>
       </c>
-      <c r="O36" s="47">
+      <c r="O36" s="46">
         <f>MIN($C$6,($I$31+$C$10*6)/O30)</f>
         <v/>
       </c>
     </row>
-    <row r="38">
+    <row r="37" ht="14.4" customHeight="1"/>
+    <row r="38" ht="14.4" customHeight="1">
       <c r="B38" s="21" t="inlineStr">
         <is>
           <t>MARKET RENT GROWTH (editable assumptions)</t>
         </is>
       </c>
-      <c r="J38" s="48" t="inlineStr">
+      <c r="J38" s="47" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="K38" s="48" t="inlineStr">
+      <c r="K38" s="47" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="L38" s="48" t="inlineStr">
+      <c r="L38" s="47" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="M38" s="48" t="inlineStr">
+      <c r="M38" s="47" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="N38" s="48" t="inlineStr">
+      <c r="N38" s="47" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="O38" s="48" t="inlineStr">
+      <c r="O38" s="47" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="14.4" customHeight="1">
       <c r="B39" s="21" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J39" s="49" t="n">
+      <c r="J39" s="48" t="n">
         <v>-0.0025</v>
       </c>
-      <c r="K39" s="49" t="n">
+      <c r="K39" s="48" t="n">
         <v>0.0175</v>
       </c>
-      <c r="L39" s="49" t="n">
+      <c r="L39" s="48" t="n">
         <v>0.0275</v>
       </c>
-      <c r="M39" s="49" t="n">
+      <c r="M39" s="48" t="n">
         <v>0.0375</v>
       </c>
-      <c r="N39" s="49" t="n">
+      <c r="N39" s="48" t="n">
         <v>0.0275</v>
       </c>
-      <c r="O39" s="49" t="n">
+      <c r="O39" s="48" t="n">
         <v>0.0175</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="14.4" customHeight="1">
       <c r="B40" s="21" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J40" s="49" t="n">
+      <c r="J40" s="48" t="n">
         <v>0.01</v>
       </c>
-      <c r="K40" s="49" t="n">
+      <c r="K40" s="48" t="n">
         <v>0.03</v>
       </c>
-      <c r="L40" s="49" t="n">
+      <c r="L40" s="48" t="n">
         <v>0.04</v>
       </c>
-      <c r="M40" s="49" t="n">
+      <c r="M40" s="48" t="n">
         <v>0.05</v>
       </c>
-      <c r="N40" s="49" t="n">
+      <c r="N40" s="48" t="n">
         <v>0.04</v>
       </c>
-      <c r="O40" s="49" t="n">
+      <c r="O40" s="48" t="n">
         <v>0.03</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="14.4" customHeight="1">
       <c r="B41" s="21" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J41" s="49" t="n">
+      <c r="J41" s="48" t="n">
         <v>0.02</v>
       </c>
-      <c r="K41" s="49" t="n">
+      <c r="K41" s="48" t="n">
         <v>0.04</v>
       </c>
-      <c r="L41" s="49" t="n">
+      <c r="L41" s="48" t="n">
         <v>0.05</v>
       </c>
-      <c r="M41" s="49" t="n">
+      <c r="M41" s="48" t="n">
         <v>0.06</v>
       </c>
-      <c r="N41" s="49" t="n">
+      <c r="N41" s="48" t="n">
         <v>0.05</v>
       </c>
-      <c r="O41" s="49" t="n">
+      <c r="O41" s="48" t="n">
         <v>0.04</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="14.4" customHeight="1">
       <c r="B42" s="21" t="inlineStr">
         <is>
-          <t>CONCESSIONS (months, editable)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
+          <t>CONCESSIONS % — forward assumption (editable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="14.4" customHeight="1">
       <c r="B43" s="21" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J43" s="49" t="n">
+      <c r="J43" s="48" t="n">
         <v>0.06</v>
       </c>
-      <c r="K43" s="49" t="n">
+      <c r="K43" s="48" t="n">
         <v>0.045</v>
       </c>
-      <c r="L43" s="49" t="n">
+      <c r="L43" s="48" t="n">
         <v>0.035</v>
       </c>
-      <c r="M43" s="49" t="n">
+      <c r="M43" s="48" t="n">
         <v>0.035</v>
       </c>
-      <c r="N43" s="49" t="n">
+      <c r="N43" s="48" t="n">
         <v>0.035</v>
       </c>
-      <c r="O43" s="49" t="n">
+      <c r="O43" s="48" t="n">
         <v>0.035</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="14.4" customHeight="1">
       <c r="B44" s="21" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J44" s="49" t="n">
+      <c r="J44" s="48" t="n">
         <v>0.03</v>
       </c>
-      <c r="K44" s="49" t="n">
+      <c r="K44" s="48" t="n">
         <v>0.015</v>
       </c>
-      <c r="L44" s="49" t="n">
+      <c r="L44" s="48" t="n">
         <v>0.005</v>
       </c>
-      <c r="M44" s="49" t="n">
+      <c r="M44" s="48" t="n">
         <v>0.005</v>
       </c>
-      <c r="N44" s="49" t="n">
+      <c r="N44" s="48" t="n">
         <v>0.005</v>
       </c>
-      <c r="O44" s="49" t="n">
+      <c r="O44" s="48" t="n">
         <v>0.005</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="14.4" customHeight="1">
       <c r="B45" s="21" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J45" s="49" t="n">
+      <c r="J45" s="48" t="n">
         <v>0.02</v>
       </c>
-      <c r="K45" s="49" t="n">
+      <c r="K45" s="48" t="n">
         <v>0.005</v>
       </c>
-      <c r="L45" s="49" t="n">
+      <c r="L45" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="M45" s="49" t="n">
+      <c r="M45" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="N45" s="49" t="n">
+      <c r="N45" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="O45" s="49" t="n">
+      <c r="O45" s="48" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="14.4" customHeight="1">
       <c r="B46" s="21" t="inlineStr">
         <is>
           <t>EFFECTIVE RENT GROWTH (derived)</t>
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="14.4" customHeight="1">
       <c r="B47" s="21" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J47" s="47">
+      <c r="J47" s="46">
         <f>(1+J39)*(1-J43)-1</f>
         <v/>
       </c>
-      <c r="K47" s="47">
+      <c r="K47" s="46">
         <f>(1+K39)*(1-K43)/(1-J43)-1</f>
         <v/>
       </c>
-      <c r="L47" s="47">
+      <c r="L47" s="46">
         <f>(1+L39)*(1-L43)/(1-K43)-1</f>
         <v/>
       </c>
-      <c r="M47" s="47">
+      <c r="M47" s="46">
         <f>(1+M39)*(1-M43)/(1-L43)-1</f>
         <v/>
       </c>
-      <c r="N47" s="47">
+      <c r="N47" s="46">
         <f>(1+N39)*(1-N43)/(1-M43)-1</f>
         <v/>
       </c>
-      <c r="O47" s="47">
+      <c r="O47" s="46">
         <f>(1+O39)*(1-O43)/(1-N43)-1</f>
         <v/>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="14.4" customHeight="1">
       <c r="B48" s="21" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J48" s="47">
+      <c r="J48" s="46">
         <f>(1+J40)*(1-J44)-1</f>
         <v/>
       </c>
-      <c r="K48" s="47">
+      <c r="K48" s="46">
         <f>(1+K40)*(1-K44)/(1-J44)-1</f>
         <v/>
       </c>
-      <c r="L48" s="47">
+      <c r="L48" s="46">
         <f>(1+L40)*(1-L44)/(1-K44)-1</f>
         <v/>
       </c>
-      <c r="M48" s="47">
+      <c r="M48" s="46">
         <f>(1+M40)*(1-M44)/(1-L44)-1</f>
         <v/>
       </c>
-      <c r="N48" s="47">
+      <c r="N48" s="46">
         <f>(1+N40)*(1-N44)/(1-M44)-1</f>
         <v/>
       </c>
-      <c r="O48" s="47">
+      <c r="O48" s="46">
         <f>(1+O40)*(1-O44)/(1-N44)-1</f>
         <v/>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="14.4" customHeight="1">
       <c r="B49" s="21" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J49" s="47">
+      <c r="J49" s="46">
         <f>(1+J41)*(1-J45)-1</f>
         <v/>
       </c>
-      <c r="K49" s="47">
+      <c r="K49" s="46">
         <f>(1+K41)*(1-K45)/(1-J45)-1</f>
         <v/>
       </c>
-      <c r="L49" s="47">
+      <c r="L49" s="46">
         <f>(1+L41)*(1-L45)/(1-K45)-1</f>
         <v/>
       </c>
-      <c r="M49" s="47">
+      <c r="M49" s="46">
         <f>(1+M41)*(1-M45)/(1-L45)-1</f>
         <v/>
       </c>
-      <c r="N49" s="47">
+      <c r="N49" s="46">
         <f>(1+N41)*(1-N45)/(1-M45)-1</f>
         <v/>
       </c>
-      <c r="O49" s="47">
+      <c r="O49" s="46">
         <f>(1+O41)*(1-O45)/(1-N45)-1</f>
         <v/>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="19" t="inlineStr">
-        <is>
-          <t>Reconciliation: UC pipeline scheduled = 0 units vs CoStar current Under Construction = 27 units.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="19" t="inlineStr">
-        <is>
-          <t>Note: as-of quarter (2026 Q2 QTD) is partial (quarter-to-date). Occupancy is point-in-time (valid); Y0 supply/absorption sums for that quarter are partial.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="B52" s="19" t="inlineStr">
-        <is>
-          <t>Historical = CoStar 5-mi TTM actuals. Forecast: inventory += UC (linked from Competitive Analysis) + proposed built this scenario; occupied += selected demand (capped at target). Yellow cells are editable.</t>
-        </is>
-      </c>
-    </row>
+    <row r="50" ht="14.4" customHeight="1"/>
+    <row r="51" ht="14.4" customHeight="1">
+      <c r="B51" s="47" t="inlineStr">
+        <is>
+          <t>▸ DETAIL: subject rent source by year &amp; reconciliation (grouped — click − to collapse)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B52" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -Y6  Q3 2019–Q2 2020</t>
+        </is>
+      </c>
+      <c r="E52" s="49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B53" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -Y5  Q3 2020–Q2 2021</t>
+        </is>
+      </c>
+      <c r="E53" s="49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B54" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -Y4  Q3 2021–Q2 2022</t>
+        </is>
+      </c>
+      <c r="E54" s="49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B55" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -Y3  Q3 2022–Q2 2023</t>
+        </is>
+      </c>
+      <c r="E55" s="49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B56" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -Y2  Q3 2023–Q2 2024</t>
+        </is>
+      </c>
+      <c r="E56" s="49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B57" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -Y1  Q3 2024–Q2 2025</t>
+        </is>
+      </c>
+      <c r="E57" s="49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B58" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Y0  Q3 2025–Q2 2026</t>
+        </is>
+      </c>
+      <c r="E58" s="49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B59" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  UC scheduled vs CoStar UC</t>
+        </is>
+      </c>
+      <c r="E59" s="49" t="inlineStr">
+        <is>
+          <t>0 / 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B60" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  As-of 2026 Q2 QTD is partial (QTD); occupancy is point-in-time, Y0 flow sums partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="14.4" customHeight="1"/>
+    <row r="62" ht="14.4" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:O2"/>

</xml_diff>